<commit_message>
Add LaTeX tables for school data in 2013 and 2014
- Created 'tabela_escolas_2013.tex' to present data on state schools with high school in Minas Gerais for 2013, including class duration and shift details.
- Created 'tabela_saida_junto.tex' to show the number of schools with 1st- and 2nd/3rd-year classes in the same shift from 2013 to 2015, along with release time statistics.
</commit_message>
<xml_diff>
--- a/output/tabela_escolas_2013.xlsx
+++ b/output/tabela_escolas_2013.xlsx
@@ -7,7 +7,8 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="escolas_2013" sheetId="1" r:id="rId1"/>
+    <sheet name="saida_junto" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,4 +473,78 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Schools with 1st- and 2nd/3rd-year classes in the same shift</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Release within 5 min: N</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>2013</v>
+      </c>
+      <c r="B2">
+        <v>1766</v>
+      </c>
+      <c r="C2">
+        <v>1687</v>
+      </c>
+      <c r="D2">
+        <v>81.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2014</v>
+      </c>
+      <c r="B3">
+        <v>1814</v>
+      </c>
+      <c r="C3">
+        <v>535</v>
+      </c>
+      <c r="D3">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>2015</v>
+      </c>
+      <c r="B4">
+        <v>1931</v>
+      </c>
+      <c r="C4">
+        <v>1763</v>
+      </c>
+      <c r="D4">
+        <v>84.90000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>